<commit_message>
add code to compare lvl 2 and 4 atc codes with drug targets
</commit_message>
<xml_diff>
--- a/LR_ANOVA_ATC_Level234.xlsx
+++ b/LR_ANOVA_ATC_Level234.xlsx
@@ -475,22 +475,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.6682033898305086</v>
+        <v>0.6758983050847458</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6649830508474576</v>
+        <v>0.6677966101694917</v>
       </c>
       <c r="E2" t="n">
-        <v>0.6900677966101694</v>
+        <v>0.6796271186440679</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5449491525423729</v>
+        <v>0.5391186440677965</v>
       </c>
       <c r="G2" t="n">
-        <v>1162.697716631235</v>
+        <v>1168.720528419339</v>
       </c>
       <c r="H2" t="n">
-        <v>9.588567216102584e-164</v>
+        <v>4.728379519944277e-164</v>
       </c>
     </row>
     <row r="3">
@@ -503,22 +503,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.6752095808383233</v>
+        <v>0.6831437125748502</v>
       </c>
       <c r="D3" t="n">
-        <v>0.680748502994012</v>
+        <v>0.6688922155688622</v>
       </c>
       <c r="E3" t="n">
-        <v>0.678562874251497</v>
+        <v>0.6832634730538922</v>
       </c>
       <c r="F3" t="n">
-        <v>0.5535329341317365</v>
+        <v>0.5563173652694612</v>
       </c>
       <c r="G3" t="n">
-        <v>1223.332095694199</v>
+        <v>1232.911302680859</v>
       </c>
       <c r="H3" t="n">
-        <v>9.023775083006992e-167</v>
+        <v>3.09030311876003e-167</v>
       </c>
     </row>
     <row r="4">
@@ -531,22 +531,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.6778797468354431</v>
+        <v>0.6656962025316456</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6799367088607595</v>
+        <v>0.680221518987342</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6830696202531644</v>
+        <v>0.6847784810126583</v>
       </c>
       <c r="F4" t="n">
-        <v>0.572246835443038</v>
+        <v>0.5705063291139241</v>
       </c>
       <c r="G4" t="n">
-        <v>845.9692507247286</v>
+        <v>728.472148597358</v>
       </c>
       <c r="H4" t="n">
-        <v>4.148129013415922e-145</v>
+        <v>1.5044865142193e-136</v>
       </c>
     </row>
     <row r="5">
@@ -559,22 +559,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.677913907284768</v>
+        <v>0.6647350993377482</v>
       </c>
       <c r="D5" t="n">
-        <v>0.675662251655629</v>
+        <v>0.6704966887417215</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6834768211920529</v>
+        <v>0.674503311258278</v>
       </c>
       <c r="F5" t="n">
-        <v>0.5695364238410595</v>
+        <v>0.5654966887417219</v>
       </c>
       <c r="G5" t="n">
-        <v>1004.848804753785</v>
+        <v>798.0560485543517</v>
       </c>
       <c r="H5" t="n">
-        <v>3.97102989400072e-155</v>
+        <v>9.382497378115046e-142</v>
       </c>
     </row>
     <row r="6">
@@ -587,22 +587,22 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.6924013157894735</v>
+        <v>0.6964473684210526</v>
       </c>
       <c r="D6" t="n">
-        <v>0.6887171052631578</v>
+        <v>0.6738157894736841</v>
       </c>
       <c r="E6" t="n">
-        <v>0.672796052631579</v>
+        <v>0.6632236842105264</v>
       </c>
       <c r="F6" t="n">
-        <v>0.5266776315789473</v>
+        <v>0.5262828947368421</v>
       </c>
       <c r="G6" t="n">
-        <v>1668.967189419673</v>
+        <v>1532.94595600719</v>
       </c>
       <c r="H6" t="n">
-        <v>1.693920492435314e-185</v>
+        <v>2.460005253900452e-180</v>
       </c>
     </row>
     <row r="7">
@@ -615,22 +615,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.7168164794007491</v>
+        <v>0.707677902621723</v>
       </c>
       <c r="D7" t="n">
-        <v>0.7197003745318352</v>
+        <v>0.7111235955056182</v>
       </c>
       <c r="E7" t="n">
-        <v>0.7112734082397004</v>
+        <v>0.7082022471910113</v>
       </c>
       <c r="F7" t="n">
-        <v>0.5579026217228464</v>
+        <v>0.5468164794007491</v>
       </c>
       <c r="G7" t="n">
-        <v>1457.408848472711</v>
+        <v>1499.301748629733</v>
       </c>
       <c r="H7" t="n">
-        <v>2.797037433293459e-177</v>
+        <v>5.421530652301393e-179</v>
       </c>
     </row>
     <row r="8">
@@ -643,22 +643,22 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.6955072463768117</v>
+        <v>0.6907971014492756</v>
       </c>
       <c r="D8" t="n">
-        <v>0.6956159420289856</v>
+        <v>0.6847101449275366</v>
       </c>
       <c r="E8" t="n">
-        <v>0.7014130434782611</v>
+        <v>0.6810869565217393</v>
       </c>
       <c r="F8" t="n">
-        <v>0.5413043478260868</v>
+        <v>0.5442028985507246</v>
       </c>
       <c r="G8" t="n">
-        <v>1679.732977496198</v>
+        <v>1168.512580973423</v>
       </c>
       <c r="H8" t="n">
-        <v>6.877678304590172e-186</v>
+        <v>4.844947855825981e-164</v>
       </c>
     </row>
     <row r="9">
@@ -671,22 +671,22 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.7121268656716417</v>
+        <v>0.7000746268656716</v>
       </c>
       <c r="D9" t="n">
-        <v>0.7122014925373135</v>
+        <v>0.7103358208955224</v>
       </c>
       <c r="E9" t="n">
-        <v>0.7047388059701493</v>
+        <v>0.703320895522388</v>
       </c>
       <c r="F9" t="n">
-        <v>0.5851119402985073</v>
+        <v>0.5866791044776118</v>
       </c>
       <c r="G9" t="n">
-        <v>768.1324925338337</v>
+        <v>747.6217068655412</v>
       </c>
       <c r="H9" t="n">
-        <v>1.443479198554364e-139</v>
+        <v>5.041405079290383e-138</v>
       </c>
     </row>
     <row r="10">
@@ -699,22 +699,22 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.6842400000000002</v>
+        <v>0.6832799999999999</v>
       </c>
       <c r="D10" t="n">
-        <v>0.6934400000000001</v>
+        <v>0.67948</v>
       </c>
       <c r="E10" t="n">
-        <v>0.6630800000000001</v>
+        <v>0.6613999999999999</v>
       </c>
       <c r="F10" t="n">
-        <v>0.5803199999999999</v>
+        <v>0.582</v>
       </c>
       <c r="G10" t="n">
-        <v>515.9931414077806</v>
+        <v>511.3902923103612</v>
       </c>
       <c r="H10" t="n">
-        <v>2.023805251347718e-117</v>
+        <v>6.171077669820094e-117</v>
       </c>
     </row>
     <row r="11">
@@ -727,22 +727,22 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.6998723404255319</v>
+        <v>0.6988936170212767</v>
       </c>
       <c r="D11" t="n">
-        <v>0.700936170212766</v>
+        <v>0.6989787234042553</v>
       </c>
       <c r="E11" t="n">
-        <v>0.6891063829787234</v>
+        <v>0.689744680851064</v>
       </c>
       <c r="F11" t="n">
-        <v>0.5947234042553191</v>
+        <v>0.5822127659574468</v>
       </c>
       <c r="G11" t="n">
-        <v>509.0235524224042</v>
+        <v>488.4736445705466</v>
       </c>
       <c r="H11" t="n">
-        <v>1.098373703736468e-116</v>
+        <v>1.805858763353032e-114</v>
       </c>
     </row>
     <row r="12">
@@ -755,22 +755,22 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.6946491228070176</v>
+        <v>0.6777192982456142</v>
       </c>
       <c r="D12" t="n">
-        <v>0.6950000000000002</v>
+        <v>0.6921052631578947</v>
       </c>
       <c r="E12" t="n">
-        <v>0.7031140350877194</v>
+        <v>0.6988157894736843</v>
       </c>
       <c r="F12" t="n">
-        <v>0.5830263157894737</v>
+        <v>0.588201754385965</v>
       </c>
       <c r="G12" t="n">
-        <v>604.1513088856071</v>
+        <v>540.6800074139782</v>
       </c>
       <c r="H12" t="n">
-        <v>4.696561061171749e-126</v>
+        <v>5.881944955558278e-120</v>
       </c>
     </row>
     <row r="13">
@@ -783,22 +783,22 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.68125</v>
+        <v>0.7123660714285713</v>
       </c>
       <c r="D13" t="n">
-        <v>0.6854910714285714</v>
+        <v>0.6876339285714285</v>
       </c>
       <c r="E13" t="n">
-        <v>0.7058928571428572</v>
+        <v>0.6976785714285714</v>
       </c>
       <c r="F13" t="n">
-        <v>0.5675892857142857</v>
+        <v>0.5672767857142857</v>
       </c>
       <c r="G13" t="n">
-        <v>939.7757320568616</v>
+        <v>859.9684322245862</v>
       </c>
       <c r="H13" t="n">
-        <v>3.282135537865571e-151</v>
+        <v>4.675251179303557e-146</v>
       </c>
     </row>
     <row r="14">
@@ -811,22 +811,22 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.6802622950819672</v>
+        <v>0.6694754098360657</v>
       </c>
       <c r="D14" t="n">
-        <v>0.6795081967213115</v>
+        <v>0.6797704918032789</v>
       </c>
       <c r="E14" t="n">
-        <v>0.6710491803278686</v>
+        <v>0.6545901639344263</v>
       </c>
       <c r="F14" t="n">
-        <v>0.5365245901639344</v>
+        <v>0.5348524590163934</v>
       </c>
       <c r="G14" t="n">
-        <v>1741.873322372194</v>
+        <v>1108.056890021586</v>
       </c>
       <c r="H14" t="n">
-        <v>4.200181348183029e-188</v>
+        <v>6.858300451817037e-161</v>
       </c>
     </row>
     <row r="15">
@@ -839,22 +839,22 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.6631553398058253</v>
+        <v>0.6561650485436894</v>
       </c>
       <c r="D15" t="n">
-        <v>0.656116504854369</v>
+        <v>0.6633009708737866</v>
       </c>
       <c r="E15" t="n">
-        <v>0.6731553398058253</v>
+        <v>0.6749029126213593</v>
       </c>
       <c r="F15" t="n">
-        <v>0.5570388349514562</v>
+        <v>0.5592718446601941</v>
       </c>
       <c r="G15" t="n">
-        <v>515.4447517559705</v>
+        <v>423.9395871321527</v>
       </c>
       <c r="H15" t="n">
-        <v>2.310285640463757e-117</v>
+        <v>5.701029436455245e-107</v>
       </c>
     </row>
     <row r="16">
@@ -867,22 +867,22 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.6462100456621005</v>
+        <v>0.6390867579908677</v>
       </c>
       <c r="D16" t="n">
-        <v>0.6431963470319634</v>
+        <v>0.6373972602739725</v>
       </c>
       <c r="E16" t="n">
-        <v>0.6679908675799087</v>
+        <v>0.6631506849315069</v>
       </c>
       <c r="F16" t="n">
-        <v>0.5599543378995433</v>
+        <v>0.5538812785388129</v>
       </c>
       <c r="G16" t="n">
-        <v>466.8126544126701</v>
+        <v>398.0278450363198</v>
       </c>
       <c r="H16" t="n">
-        <v>4.763127162060515e-112</v>
+        <v>1.073567149187739e-103</v>
       </c>
     </row>
     <row r="17">
@@ -895,22 +895,22 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.7122374429223742</v>
+        <v>0.6993150684931506</v>
       </c>
       <c r="D17" t="n">
-        <v>0.7128310502283104</v>
+        <v>0.7121917808219177</v>
       </c>
       <c r="E17" t="n">
-        <v>0.690867579908676</v>
+        <v>0.6941095890410959</v>
       </c>
       <c r="F17" t="n">
-        <v>0.6100913242009132</v>
+        <v>0.5551598173515981</v>
       </c>
       <c r="G17" t="n">
-        <v>492.7434284430469</v>
+        <v>657.9036026023573</v>
       </c>
       <c r="H17" t="n">
-        <v>6.165350775662772e-115</v>
+        <v>8.384809298344196e-131</v>
       </c>
     </row>
     <row r="18">
@@ -923,22 +923,22 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.67</v>
+        <v>0.6576076555023924</v>
       </c>
       <c r="D18" t="n">
-        <v>0.6774641148325361</v>
+        <v>0.6692822966507179</v>
       </c>
       <c r="E18" t="n">
-        <v>0.6888516746411486</v>
+        <v>0.6815311004784692</v>
       </c>
       <c r="F18" t="n">
-        <v>0.5562200956937799</v>
+        <v>0.5544976076555025</v>
       </c>
       <c r="G18" t="n">
-        <v>760.93872907025</v>
+        <v>596.8888117998347</v>
       </c>
       <c r="H18" t="n">
-        <v>4.971000734183368e-139</v>
+        <v>2.192744816196529e-125</v>
       </c>
     </row>
     <row r="19">
@@ -951,22 +951,22 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.6999069767441861</v>
+        <v>0.7086511627906975</v>
       </c>
       <c r="D19" t="n">
-        <v>0.7020000000000002</v>
+        <v>0.698</v>
       </c>
       <c r="E19" t="n">
-        <v>0.6949767441860466</v>
+        <v>0.6973953488372092</v>
       </c>
       <c r="F19" t="n">
-        <v>0.559813953488372</v>
+        <v>0.5502325581395349</v>
       </c>
       <c r="G19" t="n">
-        <v>927.6536125261226</v>
+        <v>1036.848992631338</v>
       </c>
       <c r="H19" t="n">
-        <v>1.874648163614968e-150</v>
+        <v>5.707768156770498e-157</v>
       </c>
     </row>
     <row r="20">
@@ -979,22 +979,22 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.6935960591133004</v>
+        <v>0.6979802955665023</v>
       </c>
       <c r="D20" t="n">
-        <v>0.6941871921182263</v>
+        <v>0.6917733990147782</v>
       </c>
       <c r="E20" t="n">
-        <v>0.7106403940886697</v>
+        <v>0.7089162561576353</v>
       </c>
       <c r="F20" t="n">
-        <v>0.5292118226600984</v>
+        <v>0.5316748768472904</v>
       </c>
       <c r="G20" t="n">
-        <v>1650.617601273047</v>
+        <v>1290.015007485919</v>
       </c>
       <c r="H20" t="n">
-        <v>7.972995789328821e-185</v>
+        <v>6.071751215912285e-170</v>
       </c>
     </row>
     <row r="21">
@@ -1007,22 +1007,22 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.7152083333333334</v>
+        <v>0.7084375000000001</v>
       </c>
       <c r="D21" t="n">
-        <v>0.7146354166666665</v>
+        <v>0.7156770833333335</v>
       </c>
       <c r="E21" t="n">
-        <v>0.6857812499999999</v>
+        <v>0.68265625</v>
       </c>
       <c r="F21" t="n">
-        <v>0.5365625000000001</v>
+        <v>0.5347395833333334</v>
       </c>
       <c r="G21" t="n">
-        <v>1474.549854879392</v>
+        <v>993.1681834337545</v>
       </c>
       <c r="H21" t="n">
-        <v>5.501366372012429e-178</v>
+        <v>1.926444310869916e-154</v>
       </c>
     </row>
     <row r="22">
@@ -1035,22 +1035,22 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.6897087378640776</v>
+        <v>0.6850485436893204</v>
       </c>
       <c r="D22" t="n">
-        <v>0.6904854368932039</v>
+        <v>0.6928155339805825</v>
       </c>
       <c r="E22" t="n">
-        <v>0.6838834951456311</v>
+        <v>0.6909223300970873</v>
       </c>
       <c r="F22" t="n">
-        <v>0.5616019417475728</v>
+        <v>0.5626699029126213</v>
       </c>
       <c r="G22" t="n">
-        <v>693.3526629828347</v>
+        <v>722.7689692680403</v>
       </c>
       <c r="H22" t="n">
-        <v>9.39860749618516e-134</v>
+        <v>4.199780106486351e-136</v>
       </c>
     </row>
     <row r="23">
@@ -1063,22 +1063,22 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.5984117647058822</v>
+        <v>0.6062352941176471</v>
       </c>
       <c r="D23" t="n">
-        <v>0.6044117647058823</v>
+        <v>0.5971176470588235</v>
       </c>
       <c r="E23" t="n">
-        <v>0.6455882352941177</v>
+        <v>0.635764705882353</v>
       </c>
       <c r="F23" t="n">
-        <v>0.5360588235294117</v>
+        <v>0.5272941176470588</v>
       </c>
       <c r="G23" t="n">
-        <v>312.2029179560776</v>
+        <v>318.0105783061979</v>
       </c>
       <c r="H23" t="n">
-        <v>1.756083997683842e-91</v>
+        <v>2.192792221271743e-92</v>
       </c>
     </row>
     <row r="24">
@@ -1091,22 +1091,22 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.6465816326530611</v>
+        <v>0.6560204081632652</v>
       </c>
       <c r="D24" t="n">
-        <v>0.6434183673469387</v>
+        <v>0.6385204081632654</v>
       </c>
       <c r="E24" t="n">
-        <v>0.6574489795918368</v>
+        <v>0.6474489795918368</v>
       </c>
       <c r="F24" t="n">
-        <v>0.5296428571428572</v>
+        <v>0.5299999999999999</v>
       </c>
       <c r="G24" t="n">
-        <v>669.294003959707</v>
+        <v>759.0456663884083</v>
       </c>
       <c r="H24" t="n">
-        <v>9.13425139558787e-132</v>
+        <v>6.894650777656593e-139</v>
       </c>
     </row>
     <row r="25">
@@ -1119,22 +1119,22 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.7545631067961165</v>
+        <v>0.7333495145631066</v>
       </c>
       <c r="D25" t="n">
-        <v>0.7567961165048542</v>
+        <v>0.7539320388349515</v>
       </c>
       <c r="E25" t="n">
-        <v>0.7399029126213591</v>
+        <v>0.7378640776699029</v>
       </c>
       <c r="F25" t="n">
-        <v>0.5848058252427184</v>
+        <v>0.5793203883495146</v>
       </c>
       <c r="G25" t="n">
-        <v>1396.32859266833</v>
+        <v>1065.862391136241</v>
       </c>
       <c r="H25" t="n">
-        <v>1.066784454717196e-174</v>
+        <v>1.349911821224606e-158</v>
       </c>
     </row>
     <row r="26">
@@ -1147,22 +1147,22 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0.6127659574468085</v>
+        <v>0.6098404255319148</v>
       </c>
       <c r="D26" t="n">
-        <v>0.6067553191489362</v>
+        <v>0.610531914893617</v>
       </c>
       <c r="E26" t="n">
-        <v>0.617127659574468</v>
+        <v>0.6152127659574469</v>
       </c>
       <c r="F26" t="n">
-        <v>0.5402659574468086</v>
+        <v>0.530744680851064</v>
       </c>
       <c r="G26" t="n">
-        <v>258.2818446527309</v>
+        <v>294.7019983647077</v>
       </c>
       <c r="H26" t="n">
-        <v>1.991637520807347e-82</v>
+        <v>1.112864614908677e-88</v>
       </c>
     </row>
     <row r="27">
@@ -1175,22 +1175,22 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.7151351351351352</v>
+        <v>0.7160540540540542</v>
       </c>
       <c r="D27" t="n">
-        <v>0.7160540540540542</v>
+        <v>0.6967567567567567</v>
       </c>
       <c r="E27" t="n">
-        <v>0.7204864864864864</v>
+        <v>0.7003243243243243</v>
       </c>
       <c r="F27" t="n">
-        <v>0.5207567567567568</v>
+        <v>0.5195135135135136</v>
       </c>
       <c r="G27" t="n">
-        <v>1829.049325933573</v>
+        <v>1837.229930254224</v>
       </c>
       <c r="H27" t="n">
-        <v>4.363422996834589e-191</v>
+        <v>2.327107730190732e-191</v>
       </c>
     </row>
     <row r="28">
@@ -1203,22 +1203,22 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.6676136363636364</v>
+        <v>0.6636931818181818</v>
       </c>
       <c r="D28" t="n">
-        <v>0.6722159090909092</v>
+        <v>0.6602840909090909</v>
       </c>
       <c r="E28" t="n">
-        <v>0.6289204545454545</v>
+        <v>0.6265909090909091</v>
       </c>
       <c r="F28" t="n">
-        <v>0.4888068181818182</v>
+        <v>0.4944886363636363</v>
       </c>
       <c r="G28" t="n">
-        <v>1362.88418986304</v>
+        <v>994.998146860258</v>
       </c>
       <c r="H28" t="n">
-        <v>3.065783322246379e-173</v>
+        <v>1.50252999459662e-154</v>
       </c>
     </row>
     <row r="29">
@@ -1231,22 +1231,22 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0.6793023255813952</v>
+        <v>0.6572674418604652</v>
       </c>
       <c r="D29" t="n">
-        <v>0.6880813953488374</v>
+        <v>0.6759883720930233</v>
       </c>
       <c r="E29" t="n">
-        <v>0.6925581395348839</v>
+        <v>0.6801162790697676</v>
       </c>
       <c r="F29" t="n">
-        <v>0.5384302325581396</v>
+        <v>0.5409883720930232</v>
       </c>
       <c r="G29" t="n">
-        <v>826.8664496779252</v>
+        <v>641.4836479002172</v>
       </c>
       <c r="H29" t="n">
-        <v>8.598579604489101e-144</v>
+        <v>2.17395386418817e-129</v>
       </c>
     </row>
     <row r="30">
@@ -1259,22 +1259,22 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0.6410734463276836</v>
+        <v>0.6422598870056495</v>
       </c>
       <c r="D30" t="n">
-        <v>0.6453672316384181</v>
+        <v>0.6416949152542374</v>
       </c>
       <c r="E30" t="n">
-        <v>0.6845197740112994</v>
+        <v>0.6737853107344633</v>
       </c>
       <c r="F30" t="n">
-        <v>0.4949152542372882</v>
+        <v>0.4958757062146892</v>
       </c>
       <c r="G30" t="n">
-        <v>1188.372101785567</v>
+        <v>1027.244259507349</v>
       </c>
       <c r="H30" t="n">
-        <v>4.818658902492525e-165</v>
+        <v>2.01353758830164e-156</v>
       </c>
     </row>
     <row r="31">
@@ -1287,22 +1287,22 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0.6752216748768474</v>
+        <v>0.6889655172413792</v>
       </c>
       <c r="D31" t="n">
-        <v>0.6772413793103448</v>
+        <v>0.6771428571428569</v>
       </c>
       <c r="E31" t="n">
-        <v>0.7361083743842362</v>
+        <v>0.7286699507389162</v>
       </c>
       <c r="F31" t="n">
-        <v>0.5477339901477831</v>
+        <v>0.5486206896551723</v>
       </c>
       <c r="G31" t="n">
-        <v>1276.92787340006</v>
+        <v>1203.05078199949</v>
       </c>
       <c r="H31" t="n">
-        <v>2.475597619289812e-169</v>
+        <v>8.952408760061886e-166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>